<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-03-20 17:31:36
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023</t>
+          <t>2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023</t>
+          <t>2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-03-20 21:25:05
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1802,7 +1802,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-03-21 11:18:20
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1802,7 +1802,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-04-28 10:59:29
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1757,7 +1757,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-11 16:27:59
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-13 14:41:25
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-14 22:04:56
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-15 11:50:38
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-15 16:00:24
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-16 02:28:12
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-16 09:26:08
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-16 16:52:58
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-16 17:51:43
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-16 21:51:46
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-18 11:02:06
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2025/2026, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2025/2026, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-20 20:06:39
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-21 05:05:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2022/2023, 2025/2026</t>
+          <t>2023/2024, 2025/2026, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2022/2023, 2025/2026</t>
+          <t>2023/2024, 2025/2026, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-21 09:28:38
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-22 18:51:00
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-23 11:06:04
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-23 20:41:55
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-05-23 23:52:37
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>